<commit_message>
Update DMA and USART interrupt priorities; refactor motor control functions
</commit_message>
<xml_diff>
--- a/参考资料/电气连接表.xlsx
+++ b/参考资料/电气连接表.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\STM32\Aks_SmartCar\Aks-SmartCar\参考资料\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{502D7E11-AEC8-407F-9EE3-919000680CC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DBAB492-1083-446D-B3B3-3C8FD930BB92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4470" yWindow="1750" windowWidth="19200" windowHeight="11170" xr2:uid="{1220A042-B9C9-4738-A05B-507579105497}"/>
+    <workbookView xWindow="0" yWindow="3400" windowWidth="19200" windowHeight="11170" xr2:uid="{1220A042-B9C9-4738-A05B-507579105497}"/>
   </bookViews>
   <sheets>
     <sheet name="STM32" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="157">
   <si>
     <t>舵机</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -633,6 +633,22 @@
   </si>
   <si>
     <t>PB3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>右前</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>左前</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>右后</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>左后</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -952,6 +968,57 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -961,15 +1028,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -981,39 +1039,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1022,15 +1047,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1372,16 +1388,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="7" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="48" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
@@ -1416,22 +1432,24 @@
       <c r="B3" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="C3" s="37" t="s">
+      <c r="C3" s="51" t="s">
         <v>118</v>
       </c>
       <c r="D3" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="43" t="s">
+      <c r="E3" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="44" t="s">
+      <c r="F3" s="34" t="s">
         <v>17</v>
       </c>
       <c r="G3" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="12"/>
+      <c r="H3" s="12" t="s">
+        <v>153</v>
+      </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="26" t="s">
@@ -1440,16 +1458,18 @@
       <c r="B4" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="C4" s="38"/>
+      <c r="C4" s="52"/>
       <c r="D4" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="43"/>
-      <c r="F4" s="44"/>
+      <c r="E4" s="37"/>
+      <c r="F4" s="34"/>
       <c r="G4" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="H4" s="12"/>
+      <c r="H4" s="12" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="s">
@@ -1458,14 +1478,14 @@
       <c r="B5" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="34" t="s">
+      <c r="C5" s="45" t="s">
         <v>117</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="43"/>
-      <c r="F5" s="44"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="34"/>
       <c r="G5" s="12" t="s">
         <v>13</v>
       </c>
@@ -1478,12 +1498,12 @@
       <c r="B6" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="35"/>
+      <c r="C6" s="46"/>
       <c r="D6" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="43"/>
-      <c r="F6" s="44"/>
+      <c r="E6" s="37"/>
+      <c r="F6" s="34"/>
       <c r="G6" s="12" t="s">
         <v>43</v>
       </c>
@@ -1496,12 +1516,12 @@
       <c r="B7" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="35"/>
+      <c r="C7" s="46"/>
       <c r="D7" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="43"/>
-      <c r="F7" s="44"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="34"/>
       <c r="G7" s="12" t="s">
         <v>15</v>
       </c>
@@ -1514,12 +1534,12 @@
       <c r="B8" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="36"/>
+      <c r="C8" s="47"/>
       <c r="D8" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="43"/>
-      <c r="F8" s="44"/>
+      <c r="E8" s="37"/>
+      <c r="F8" s="34"/>
       <c r="G8" s="12" t="s">
         <v>16</v>
       </c>
@@ -1532,22 +1552,24 @@
       <c r="B9" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="C9" s="37" t="s">
+      <c r="C9" s="51" t="s">
         <v>118</v>
       </c>
       <c r="D9" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="43" t="s">
+      <c r="E9" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="44" t="s">
+      <c r="F9" s="34" t="s">
         <v>18</v>
       </c>
       <c r="G9" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="H9" s="12"/>
+      <c r="H9" s="12" t="s">
+        <v>155</v>
+      </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="26" t="s">
@@ -1556,16 +1578,18 @@
       <c r="B10" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="C10" s="38"/>
+      <c r="C10" s="52"/>
       <c r="D10" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="E10" s="43"/>
-      <c r="F10" s="44"/>
+      <c r="E10" s="37"/>
+      <c r="F10" s="34"/>
       <c r="G10" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="H10" s="12"/>
+      <c r="H10" s="12" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="13" t="s">
@@ -1574,14 +1598,14 @@
       <c r="B11" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="34" t="s">
+      <c r="C11" s="45" t="s">
         <v>117</v>
       </c>
       <c r="D11" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E11" s="43"/>
-      <c r="F11" s="44"/>
+      <c r="E11" s="37"/>
+      <c r="F11" s="34"/>
       <c r="G11" s="12" t="s">
         <v>13</v>
       </c>
@@ -1594,12 +1618,12 @@
       <c r="B12" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="35"/>
+      <c r="C12" s="46"/>
       <c r="D12" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="43"/>
-      <c r="F12" s="44"/>
+      <c r="E12" s="37"/>
+      <c r="F12" s="34"/>
       <c r="G12" s="12" t="s">
         <v>14</v>
       </c>
@@ -1612,12 +1636,12 @@
       <c r="B13" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="35"/>
+      <c r="C13" s="46"/>
       <c r="D13" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E13" s="43"/>
-      <c r="F13" s="44"/>
+      <c r="E13" s="37"/>
+      <c r="F13" s="34"/>
       <c r="G13" s="12" t="s">
         <v>15</v>
       </c>
@@ -1630,12 +1654,12 @@
       <c r="B14" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="36"/>
+      <c r="C14" s="47"/>
       <c r="D14" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E14" s="43"/>
-      <c r="F14" s="44"/>
+      <c r="E14" s="37"/>
+      <c r="F14" s="34"/>
       <c r="G14" s="12" t="s">
         <v>16</v>
       </c>
@@ -1648,25 +1672,25 @@
       <c r="B15" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="C15" s="39" t="s">
+      <c r="C15" s="53" t="s">
         <v>120</v>
       </c>
       <c r="D15" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="E15" s="33" t="s">
+      <c r="E15" s="50" t="s">
         <v>82</v>
       </c>
-      <c r="F15" s="32" t="s">
+      <c r="F15" s="49" t="s">
         <v>60</v>
       </c>
       <c r="G15" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="H15" s="52" t="s">
+      <c r="H15" s="55" t="s">
         <v>124</v>
       </c>
-      <c r="I15" s="57"/>
+      <c r="I15" s="33"/>
     </row>
     <row r="16" spans="1:9" s="22" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="24" t="s">
@@ -1675,17 +1699,17 @@
       <c r="B16" s="24" t="s">
         <v>132</v>
       </c>
-      <c r="C16" s="40"/>
+      <c r="C16" s="54"/>
       <c r="D16" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="E16" s="33"/>
-      <c r="F16" s="32"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="49"/>
       <c r="G16" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="H16" s="53"/>
-      <c r="I16" s="57"/>
+      <c r="H16" s="56"/>
+      <c r="I16" s="33"/>
     </row>
     <row r="17" spans="1:9" s="22" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="24" t="s">
@@ -1694,20 +1718,20 @@
       <c r="B17" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="C17" s="39" t="s">
+      <c r="C17" s="53" t="s">
         <v>121</v>
       </c>
       <c r="D17" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="E17" s="33"/>
-      <c r="F17" s="32" t="s">
+      <c r="E17" s="50"/>
+      <c r="F17" s="49" t="s">
         <v>61</v>
       </c>
       <c r="G17" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="H17" s="53"/>
+      <c r="H17" s="56"/>
     </row>
     <row r="18" spans="1:9" s="22" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="24" t="s">
@@ -1716,16 +1740,16 @@
       <c r="B18" s="24" t="s">
         <v>128</v>
       </c>
-      <c r="C18" s="40"/>
+      <c r="C18" s="54"/>
       <c r="D18" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="E18" s="33"/>
-      <c r="F18" s="32"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="49"/>
       <c r="G18" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="H18" s="53"/>
+      <c r="H18" s="56"/>
     </row>
     <row r="19" spans="1:9" s="22" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="24" t="s">
@@ -1734,20 +1758,20 @@
       <c r="B19" s="24" t="s">
         <v>80</v>
       </c>
-      <c r="C19" s="39" t="s">
+      <c r="C19" s="53" t="s">
         <v>127</v>
       </c>
       <c r="D19" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="E19" s="33"/>
-      <c r="F19" s="32" t="s">
+      <c r="E19" s="50"/>
+      <c r="F19" s="49" t="s">
         <v>62</v>
       </c>
       <c r="G19" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="H19" s="53"/>
+      <c r="H19" s="56"/>
     </row>
     <row r="20" spans="1:9" s="22" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="24" t="s">
@@ -1756,16 +1780,16 @@
       <c r="B20" s="24" t="s">
         <v>81</v>
       </c>
-      <c r="C20" s="40"/>
+      <c r="C20" s="54"/>
       <c r="D20" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="E20" s="33"/>
-      <c r="F20" s="32"/>
+      <c r="E20" s="50"/>
+      <c r="F20" s="49"/>
       <c r="G20" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="H20" s="53"/>
+      <c r="H20" s="56"/>
     </row>
     <row r="21" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="24" t="s">
@@ -1774,21 +1798,21 @@
       <c r="B21" s="24" t="s">
         <v>74</v>
       </c>
-      <c r="C21" s="39" t="s">
+      <c r="C21" s="53" t="s">
         <v>126</v>
       </c>
       <c r="D21" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="E21" s="33"/>
-      <c r="F21" s="32" t="s">
+      <c r="E21" s="50"/>
+      <c r="F21" s="49" t="s">
         <v>63</v>
       </c>
       <c r="G21" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="H21" s="53"/>
-      <c r="I21" s="57"/>
+      <c r="H21" s="56"/>
+      <c r="I21" s="33"/>
     </row>
     <row r="22" spans="1:9" s="22" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="24" t="s">
@@ -1797,17 +1821,17 @@
       <c r="B22" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="C22" s="40"/>
+      <c r="C22" s="54"/>
       <c r="D22" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="E22" s="33"/>
-      <c r="F22" s="32"/>
+      <c r="E22" s="50"/>
+      <c r="F22" s="49"/>
       <c r="G22" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="H22" s="54"/>
-      <c r="I22" s="57"/>
+      <c r="H22" s="57"/>
+      <c r="I22" s="33"/>
     </row>
     <row r="23" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="13" t="s">
@@ -1822,10 +1846,10 @@
       <c r="D23" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E23" s="43" t="s">
+      <c r="E23" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="F23" s="44" t="s">
+      <c r="F23" s="34" t="s">
         <v>2</v>
       </c>
       <c r="G23" s="12" t="s">
@@ -1846,8 +1870,8 @@
       <c r="D24" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="E24" s="43"/>
-      <c r="F24" s="44"/>
+      <c r="E24" s="37"/>
+      <c r="F24" s="34"/>
       <c r="G24" s="12" t="s">
         <v>34</v>
       </c>
@@ -1866,8 +1890,8 @@
       <c r="D25" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E25" s="43"/>
-      <c r="F25" s="44" t="s">
+      <c r="E25" s="37"/>
+      <c r="F25" s="34" t="s">
         <v>3</v>
       </c>
       <c r="G25" s="12" t="s">
@@ -1888,8 +1912,8 @@
       <c r="D26" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="E26" s="43"/>
-      <c r="F26" s="44"/>
+      <c r="E26" s="37"/>
+      <c r="F26" s="34"/>
       <c r="G26" s="12" t="s">
         <v>34</v>
       </c>
@@ -1908,8 +1932,8 @@
       <c r="D27" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E27" s="43"/>
-      <c r="F27" s="44" t="s">
+      <c r="E27" s="37"/>
+      <c r="F27" s="34" t="s">
         <v>4</v>
       </c>
       <c r="G27" s="12" t="s">
@@ -1930,8 +1954,8 @@
       <c r="D28" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="E28" s="43"/>
-      <c r="F28" s="44"/>
+      <c r="E28" s="37"/>
+      <c r="F28" s="34"/>
       <c r="G28" s="12" t="s">
         <v>34</v>
       </c>
@@ -1944,22 +1968,22 @@
       <c r="B29" s="25" t="s">
         <v>134</v>
       </c>
-      <c r="C29" s="55" t="s">
+      <c r="C29" s="31" t="s">
         <v>136</v>
       </c>
       <c r="D29" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="E29" s="47" t="s">
+      <c r="E29" s="40" t="s">
         <v>55</v>
       </c>
-      <c r="F29" s="46" t="s">
+      <c r="F29" s="39" t="s">
         <v>54</v>
       </c>
       <c r="G29" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="H29" s="44" t="s">
+      <c r="H29" s="34" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1970,16 +1994,16 @@
       <c r="B30" s="25" t="s">
         <v>133</v>
       </c>
-      <c r="C30" s="56"/>
+      <c r="C30" s="32"/>
       <c r="D30" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="E30" s="47"/>
-      <c r="F30" s="46"/>
+      <c r="E30" s="40"/>
+      <c r="F30" s="39"/>
       <c r="G30" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="H30" s="44"/>
+      <c r="H30" s="34"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="27" t="s">
@@ -1994,7 +2018,7 @@
       <c r="D31" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="E31" s="45" t="s">
+      <c r="E31" s="38" t="s">
         <v>0</v>
       </c>
       <c r="F31" s="28" t="s">
@@ -2018,7 +2042,7 @@
       <c r="D32" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="E32" s="45"/>
+      <c r="E32" s="38"/>
       <c r="F32" s="28" t="s">
         <v>48</v>
       </c>
@@ -2034,16 +2058,16 @@
       <c r="B33" s="20" t="s">
         <v>137</v>
       </c>
-      <c r="C33" s="48" t="s">
+      <c r="C33" s="41" t="s">
         <v>135</v>
       </c>
       <c r="D33" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="E33" s="48" t="s">
+      <c r="E33" s="41" t="s">
         <v>115</v>
       </c>
-      <c r="F33" s="50" t="s">
+      <c r="F33" s="43" t="s">
         <v>114</v>
       </c>
       <c r="G33" s="19" t="s">
@@ -2058,12 +2082,12 @@
       <c r="B34" s="20" t="s">
         <v>138</v>
       </c>
-      <c r="C34" s="49"/>
+      <c r="C34" s="42"/>
       <c r="D34" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="E34" s="49"/>
-      <c r="F34" s="51"/>
+      <c r="E34" s="42"/>
+      <c r="F34" s="44"/>
       <c r="G34" s="19" t="s">
         <v>58</v>
       </c>
@@ -2075,24 +2099,24 @@
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A36" s="41" t="s">
+      <c r="A36" s="35" t="s">
         <v>123</v>
       </c>
-      <c r="B36" s="42"/>
-      <c r="C36" s="42"/>
-      <c r="D36" s="42"/>
-      <c r="E36" s="42"/>
-      <c r="F36" s="42"/>
+      <c r="B36" s="36"/>
+      <c r="C36" s="36"/>
+      <c r="D36" s="36"/>
+      <c r="E36" s="36"/>
+      <c r="F36" s="36"/>
       <c r="G36" s="5"/>
       <c r="H36" s="5"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A37" s="42"/>
-      <c r="B37" s="42"/>
-      <c r="C37" s="42"/>
-      <c r="D37" s="42"/>
-      <c r="E37" s="42"/>
-      <c r="F37" s="42"/>
+      <c r="A37" s="36"/>
+      <c r="B37" s="36"/>
+      <c r="C37" s="36"/>
+      <c r="D37" s="36"/>
+      <c r="E37" s="36"/>
+      <c r="F37" s="36"/>
       <c r="G37" s="5"/>
       <c r="H37" s="5"/>
     </row>
@@ -2118,24 +2142,6 @@
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="H29:H30"/>
-    <mergeCell ref="A36:F37"/>
-    <mergeCell ref="E3:E8"/>
-    <mergeCell ref="F3:F8"/>
-    <mergeCell ref="E9:E14"/>
-    <mergeCell ref="F9:F14"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="E23:E28"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="F33:F34"/>
     <mergeCell ref="C5:C8"/>
     <mergeCell ref="C33:C34"/>
     <mergeCell ref="A1:H1"/>
@@ -2152,6 +2158,24 @@
     <mergeCell ref="C19:C20"/>
     <mergeCell ref="C21:C22"/>
     <mergeCell ref="H15:H22"/>
+    <mergeCell ref="E3:E8"/>
+    <mergeCell ref="F3:F8"/>
+    <mergeCell ref="E9:E14"/>
+    <mergeCell ref="F9:F14"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="E23:E28"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="H29:H30"/>
+    <mergeCell ref="A36:F37"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="F33:F34"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2175,14 +2199,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="48" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
@@ -2205,16 +2229,16 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="43">
+      <c r="A3" s="37">
         <v>1</v>
       </c>
       <c r="B3" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="C3" s="43" t="s">
+      <c r="C3" s="37" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="43" t="s">
+      <c r="D3" s="37" t="s">
         <v>7</v>
       </c>
       <c r="E3" s="12" t="s">
@@ -2225,26 +2249,26 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="43"/>
+      <c r="A4" s="37"/>
       <c r="B4" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="C4" s="43"/>
-      <c r="D4" s="43"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="37"/>
       <c r="E4" s="12" t="s">
         <v>27</v>
       </c>
       <c r="F4" s="58"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="43"/>
+      <c r="A5" s="37"/>
       <c r="B5" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="C5" s="43" t="s">
+      <c r="C5" s="37" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="43" t="s">
+      <c r="D5" s="37" t="s">
         <v>7</v>
       </c>
       <c r="E5" s="12" t="s">
@@ -2255,28 +2279,28 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="43"/>
+      <c r="A6" s="37"/>
       <c r="B6" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="C6" s="43"/>
-      <c r="D6" s="43"/>
+      <c r="C6" s="37"/>
+      <c r="D6" s="37"/>
       <c r="E6" s="12" t="s">
         <v>27</v>
       </c>
       <c r="F6" s="58"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="43">
+      <c r="A7" s="37">
         <v>2</v>
       </c>
       <c r="B7" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="C7" s="43" t="s">
+      <c r="C7" s="37" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="43" t="s">
+      <c r="D7" s="37" t="s">
         <v>7</v>
       </c>
       <c r="E7" s="12" t="s">
@@ -2287,26 +2311,26 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="43"/>
+      <c r="A8" s="37"/>
       <c r="B8" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="C8" s="43"/>
-      <c r="D8" s="43"/>
+      <c r="C8" s="37"/>
+      <c r="D8" s="37"/>
       <c r="E8" s="12" t="s">
         <v>27</v>
       </c>
       <c r="F8" s="58"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="43"/>
+      <c r="A9" s="37"/>
       <c r="B9" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="C9" s="43" t="s">
+      <c r="C9" s="37" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="43" t="s">
+      <c r="D9" s="37" t="s">
         <v>7</v>
       </c>
       <c r="E9" s="12" t="s">
@@ -2317,12 +2341,12 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="43"/>
+      <c r="A10" s="37"/>
       <c r="B10" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="C10" s="43"/>
-      <c r="D10" s="43"/>
+      <c r="C10" s="37"/>
+      <c r="D10" s="37"/>
       <c r="E10" s="12" t="s">
         <v>27</v>
       </c>
@@ -2366,13 +2390,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="48" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
       <c r="F1" s="6"/>
       <c r="G1" s="6"/>
     </row>

</xml_diff>

<commit_message>
Refactor motor speed handling; change speed variables to float and update initialization for improved precision Finish 4 wheels speed reading task
</commit_message>
<xml_diff>
--- a/参考资料/电气连接表.xlsx
+++ b/参考资料/电气连接表.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\STM32\Aks_SmartCar\Aks-SmartCar\参考资料\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DBAB492-1083-446D-B3B3-3C8FD930BB92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AADD7727-6FA6-4631-8601-2633AAA7A1C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="3400" windowWidth="19200" windowHeight="11170" xr2:uid="{1220A042-B9C9-4738-A05B-507579105497}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{1220A042-B9C9-4738-A05B-507579105497}"/>
   </bookViews>
   <sheets>
     <sheet name="STM32" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="157">
   <si>
     <t>舵机</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -265,22 +265,6 @@
   </si>
   <si>
     <t>PA2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>JGB37-520电机编码器1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>JGB37-520电机编码器2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>JGB37-520电机编码器3</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>JGB37-520电机编码器4</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -649,6 +633,22 @@
   </si>
   <si>
     <t>左后</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>JGB37-520电机编码器1LF</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>JGB37-520电机编码器2RF</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>JGB37-520电机编码器3LB</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>JGB37-520电机编码器4RB</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -790,7 +790,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -868,13 +868,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -968,6 +990,66 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -977,78 +1059,18 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1057,6 +1079,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1388,16 +1422,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="7" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
@@ -1407,7 +1441,7 @@
         <v>19</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D2" s="9" t="s">
         <v>8</v>
@@ -1430,25 +1464,25 @@
         <v>23</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>66</v>
-      </c>
-      <c r="C3" s="51" t="s">
-        <v>118</v>
+        <v>62</v>
+      </c>
+      <c r="C3" s="39" t="s">
+        <v>114</v>
       </c>
       <c r="D3" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="37" t="s">
+      <c r="E3" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="34" t="s">
+      <c r="F3" s="47" t="s">
         <v>17</v>
       </c>
       <c r="G3" s="12" t="s">
         <v>11</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -1456,19 +1490,19 @@
         <v>24</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="C4" s="52"/>
+        <v>63</v>
+      </c>
+      <c r="C4" s="40"/>
       <c r="D4" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="37"/>
-      <c r="F4" s="34"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="47"/>
       <c r="G4" s="12" t="s">
         <v>12</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -1478,18 +1512,20 @@
       <c r="B5" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="45" t="s">
-        <v>117</v>
+      <c r="C5" s="31" t="s">
+        <v>113</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="37"/>
-      <c r="F5" s="34"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="47"/>
       <c r="G5" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="12"/>
+      <c r="H5" s="61" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
@@ -1498,16 +1534,16 @@
       <c r="B6" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="46"/>
+      <c r="C6" s="32"/>
       <c r="D6" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="37"/>
-      <c r="F6" s="34"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="47"/>
       <c r="G6" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="H6" s="12"/>
+      <c r="H6" s="62"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
@@ -1516,16 +1552,18 @@
       <c r="B7" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="46"/>
+      <c r="C7" s="32"/>
       <c r="D7" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="37"/>
-      <c r="F7" s="34"/>
+      <c r="E7" s="46"/>
+      <c r="F7" s="47"/>
       <c r="G7" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="12"/>
+      <c r="H7" s="61" t="s">
+        <v>150</v>
+      </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
@@ -1534,41 +1572,41 @@
       <c r="B8" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="47"/>
+      <c r="C8" s="33"/>
       <c r="D8" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="37"/>
-      <c r="F8" s="34"/>
+      <c r="E8" s="46"/>
+      <c r="F8" s="47"/>
       <c r="G8" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="H8" s="12"/>
+      <c r="H8" s="62"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="26" t="s">
         <v>22</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>68</v>
-      </c>
-      <c r="C9" s="51" t="s">
-        <v>118</v>
+        <v>64</v>
+      </c>
+      <c r="C9" s="39" t="s">
+        <v>114</v>
       </c>
       <c r="D9" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="37" t="s">
+      <c r="E9" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="34" t="s">
+      <c r="F9" s="47" t="s">
         <v>18</v>
       </c>
       <c r="G9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -1576,19 +1614,19 @@
         <v>25</v>
       </c>
       <c r="B10" s="26" t="s">
-        <v>69</v>
-      </c>
-      <c r="C10" s="52"/>
+        <v>65</v>
+      </c>
+      <c r="C10" s="40"/>
       <c r="D10" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="E10" s="37"/>
-      <c r="F10" s="34"/>
+      <c r="E10" s="46"/>
+      <c r="F10" s="47"/>
       <c r="G10" s="12" t="s">
         <v>12</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
@@ -1598,18 +1636,20 @@
       <c r="B11" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="45" t="s">
-        <v>117</v>
+      <c r="C11" s="31" t="s">
+        <v>113</v>
       </c>
       <c r="D11" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E11" s="37"/>
-      <c r="F11" s="34"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="47"/>
       <c r="G11" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H11" s="12"/>
+      <c r="H11" s="63" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="s">
@@ -1618,16 +1658,16 @@
       <c r="B12" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="46"/>
+      <c r="C12" s="32"/>
       <c r="D12" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="37"/>
-      <c r="F12" s="34"/>
+      <c r="E12" s="46"/>
+      <c r="F12" s="47"/>
       <c r="G12" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H12" s="12"/>
+      <c r="H12" s="64"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="13" t="s">
@@ -1636,16 +1676,18 @@
       <c r="B13" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="46"/>
+      <c r="C13" s="32"/>
       <c r="D13" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E13" s="37"/>
-      <c r="F13" s="34"/>
+      <c r="E13" s="46"/>
+      <c r="F13" s="47"/>
       <c r="G13" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H13" s="12"/>
+      <c r="H13" s="61" t="s">
+        <v>152</v>
+      </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="13" t="s">
@@ -1654,202 +1696,202 @@
       <c r="B14" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="47"/>
+      <c r="C14" s="33"/>
       <c r="D14" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E14" s="37"/>
-      <c r="F14" s="34"/>
+      <c r="E14" s="46"/>
+      <c r="F14" s="47"/>
       <c r="G14" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="H14" s="12"/>
+      <c r="H14" s="62"/>
     </row>
     <row r="15" spans="1:9" s="22" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="24" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B15" s="24" t="s">
-        <v>70</v>
-      </c>
-      <c r="C15" s="53" t="s">
-        <v>120</v>
+        <v>66</v>
+      </c>
+      <c r="C15" s="41" t="s">
+        <v>116</v>
       </c>
       <c r="D15" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="E15" s="50" t="s">
-        <v>82</v>
-      </c>
-      <c r="F15" s="49" t="s">
+      <c r="E15" s="38" t="s">
+        <v>78</v>
+      </c>
+      <c r="F15" s="37" t="s">
+        <v>153</v>
+      </c>
+      <c r="G15" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="G15" s="21" t="s">
-        <v>64</v>
-      </c>
-      <c r="H15" s="55" t="s">
-        <v>124</v>
-      </c>
-      <c r="I15" s="33"/>
+      <c r="H15" s="43" t="s">
+        <v>120</v>
+      </c>
+      <c r="I15" s="53"/>
     </row>
     <row r="16" spans="1:9" s="22" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="24" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B16" s="24" t="s">
-        <v>132</v>
-      </c>
-      <c r="C16" s="54"/>
+        <v>128</v>
+      </c>
+      <c r="C16" s="42"/>
       <c r="D16" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="E16" s="50"/>
-      <c r="F16" s="49"/>
+      <c r="E16" s="38"/>
+      <c r="F16" s="37"/>
       <c r="G16" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="H16" s="56"/>
-      <c r="I16" s="33"/>
+        <v>61</v>
+      </c>
+      <c r="H16" s="44"/>
+      <c r="I16" s="53"/>
     </row>
     <row r="17" spans="1:9" s="22" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="24" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B17" s="24" t="s">
-        <v>77</v>
-      </c>
-      <c r="C17" s="53" t="s">
-        <v>121</v>
+        <v>73</v>
+      </c>
+      <c r="C17" s="41" t="s">
+        <v>117</v>
       </c>
       <c r="D17" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="E17" s="50"/>
-      <c r="F17" s="49" t="s">
-        <v>61</v>
+      <c r="E17" s="38"/>
+      <c r="F17" s="37" t="s">
+        <v>154</v>
       </c>
       <c r="G17" s="21" t="s">
-        <v>64</v>
-      </c>
-      <c r="H17" s="56"/>
+        <v>60</v>
+      </c>
+      <c r="H17" s="44"/>
     </row>
     <row r="18" spans="1:9" s="22" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="24" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B18" s="24" t="s">
-        <v>128</v>
-      </c>
-      <c r="C18" s="54"/>
+        <v>124</v>
+      </c>
+      <c r="C18" s="42"/>
       <c r="D18" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="E18" s="50"/>
-      <c r="F18" s="49"/>
+      <c r="E18" s="38"/>
+      <c r="F18" s="37"/>
       <c r="G18" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="H18" s="56"/>
+        <v>61</v>
+      </c>
+      <c r="H18" s="44"/>
     </row>
     <row r="19" spans="1:9" s="22" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="24" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B19" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="C19" s="53" t="s">
-        <v>127</v>
+        <v>76</v>
+      </c>
+      <c r="C19" s="41" t="s">
+        <v>123</v>
       </c>
       <c r="D19" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="E19" s="50"/>
-      <c r="F19" s="49" t="s">
-        <v>62</v>
+      <c r="E19" s="38"/>
+      <c r="F19" s="37" t="s">
+        <v>155</v>
       </c>
       <c r="G19" s="21" t="s">
-        <v>64</v>
-      </c>
-      <c r="H19" s="56"/>
+        <v>60</v>
+      </c>
+      <c r="H19" s="44"/>
     </row>
     <row r="20" spans="1:9" s="22" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="24" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B20" s="24" t="s">
-        <v>81</v>
-      </c>
-      <c r="C20" s="54"/>
+        <v>77</v>
+      </c>
+      <c r="C20" s="42"/>
       <c r="D20" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="E20" s="50"/>
-      <c r="F20" s="49"/>
+      <c r="E20" s="38"/>
+      <c r="F20" s="37"/>
       <c r="G20" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="H20" s="56"/>
+        <v>61</v>
+      </c>
+      <c r="H20" s="44"/>
     </row>
     <row r="21" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="24" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B21" s="24" t="s">
-        <v>74</v>
-      </c>
-      <c r="C21" s="53" t="s">
-        <v>126</v>
+        <v>70</v>
+      </c>
+      <c r="C21" s="41" t="s">
+        <v>122</v>
       </c>
       <c r="D21" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="E21" s="50"/>
-      <c r="F21" s="49" t="s">
-        <v>63</v>
+      <c r="E21" s="38"/>
+      <c r="F21" s="37" t="s">
+        <v>156</v>
       </c>
       <c r="G21" s="21" t="s">
-        <v>64</v>
-      </c>
-      <c r="H21" s="56"/>
-      <c r="I21" s="33"/>
+        <v>60</v>
+      </c>
+      <c r="H21" s="44"/>
+      <c r="I21" s="53"/>
     </row>
     <row r="22" spans="1:9" s="22" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="24" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B22" s="24" t="s">
-        <v>75</v>
-      </c>
-      <c r="C22" s="54"/>
+        <v>71</v>
+      </c>
+      <c r="C22" s="42"/>
       <c r="D22" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="E22" s="50"/>
-      <c r="F22" s="49"/>
+      <c r="E22" s="38"/>
+      <c r="F22" s="37"/>
       <c r="G22" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="H22" s="57"/>
-      <c r="I22" s="33"/>
+        <v>61</v>
+      </c>
+      <c r="H22" s="45"/>
+      <c r="I22" s="53"/>
     </row>
     <row r="23" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="13" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="B23" s="13" t="s">
         <v>44</v>
       </c>
       <c r="C23" s="30" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D23" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E23" s="37" t="s">
+      <c r="E23" s="46" t="s">
         <v>45</v>
       </c>
-      <c r="F23" s="34" t="s">
+      <c r="F23" s="47" t="s">
         <v>2</v>
       </c>
       <c r="G23" s="12" t="s">
@@ -1859,19 +1901,19 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="26" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B24" s="26" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C24" s="29" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="D24" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="E24" s="37"/>
-      <c r="F24" s="34"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="47"/>
       <c r="G24" s="12" t="s">
         <v>34</v>
       </c>
@@ -1879,19 +1921,19 @@
     </row>
     <row r="25" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="13" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B25" s="13" t="s">
         <v>44</v>
       </c>
       <c r="C25" s="30" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D25" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E25" s="37"/>
-      <c r="F25" s="34" t="s">
+      <c r="E25" s="46"/>
+      <c r="F25" s="47" t="s">
         <v>3</v>
       </c>
       <c r="G25" s="12" t="s">
@@ -1901,19 +1943,19 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="26" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B26" s="26" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C26" s="29" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="D26" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="E26" s="37"/>
-      <c r="F26" s="34"/>
+      <c r="E26" s="46"/>
+      <c r="F26" s="47"/>
       <c r="G26" s="12" t="s">
         <v>34</v>
       </c>
@@ -1921,19 +1963,19 @@
     </row>
     <row r="27" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="13" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B27" s="13" t="s">
         <v>44</v>
       </c>
       <c r="C27" s="30" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D27" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E27" s="37"/>
-      <c r="F27" s="34" t="s">
+      <c r="E27" s="46"/>
+      <c r="F27" s="47" t="s">
         <v>4</v>
       </c>
       <c r="G27" s="12" t="s">
@@ -1946,16 +1988,16 @@
         <v>59</v>
       </c>
       <c r="B28" s="26" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C28" s="29" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="D28" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="E28" s="37"/>
-      <c r="F28" s="34"/>
+      <c r="E28" s="46"/>
+      <c r="F28" s="47"/>
       <c r="G28" s="12" t="s">
         <v>34</v>
       </c>
@@ -1963,62 +2005,62 @@
     </row>
     <row r="29" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="25" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="B29" s="25" t="s">
-        <v>134</v>
-      </c>
-      <c r="C29" s="31" t="s">
-        <v>136</v>
+        <v>130</v>
+      </c>
+      <c r="C29" s="51" t="s">
+        <v>132</v>
       </c>
       <c r="D29" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="E29" s="40" t="s">
+      <c r="E29" s="50" t="s">
         <v>55</v>
       </c>
-      <c r="F29" s="39" t="s">
+      <c r="F29" s="49" t="s">
         <v>54</v>
       </c>
       <c r="G29" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="H29" s="34" t="s">
+      <c r="H29" s="47" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="30" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="25" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B30" s="25" t="s">
-        <v>133</v>
-      </c>
-      <c r="C30" s="32"/>
+        <v>129</v>
+      </c>
+      <c r="C30" s="52"/>
       <c r="D30" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="E30" s="40"/>
-      <c r="F30" s="39"/>
+      <c r="E30" s="50"/>
+      <c r="F30" s="49"/>
       <c r="G30" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="H30" s="34"/>
+      <c r="H30" s="47"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="27" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="B31" s="27" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="D31" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="E31" s="38" t="s">
+      <c r="E31" s="48" t="s">
         <v>0</v>
       </c>
       <c r="F31" s="28" t="s">
@@ -2031,18 +2073,18 @@
     </row>
     <row r="32" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="27" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B32" s="27" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C32" s="27" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="D32" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="E32" s="38"/>
+      <c r="E32" s="48"/>
       <c r="F32" s="28" t="s">
         <v>48</v>
       </c>
@@ -2053,22 +2095,22 @@
     </row>
     <row r="33" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="20" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B33" s="20" t="s">
-        <v>137</v>
-      </c>
-      <c r="C33" s="41" t="s">
-        <v>135</v>
+        <v>133</v>
+      </c>
+      <c r="C33" s="34" t="s">
+        <v>131</v>
       </c>
       <c r="D33" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="E33" s="41" t="s">
-        <v>115</v>
-      </c>
-      <c r="F33" s="43" t="s">
-        <v>114</v>
+      <c r="E33" s="34" t="s">
+        <v>111</v>
+      </c>
+      <c r="F33" s="56" t="s">
+        <v>110</v>
       </c>
       <c r="G33" s="19" t="s">
         <v>57</v>
@@ -2077,17 +2119,17 @@
     </row>
     <row r="34" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="20" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>138</v>
-      </c>
-      <c r="C34" s="42"/>
+        <v>134</v>
+      </c>
+      <c r="C34" s="35"/>
       <c r="D34" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="E34" s="42"/>
-      <c r="F34" s="44"/>
+      <c r="E34" s="35"/>
+      <c r="F34" s="57"/>
       <c r="G34" s="19" t="s">
         <v>58</v>
       </c>
@@ -2099,24 +2141,24 @@
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A36" s="35" t="s">
-        <v>123</v>
-      </c>
-      <c r="B36" s="36"/>
-      <c r="C36" s="36"/>
-      <c r="D36" s="36"/>
-      <c r="E36" s="36"/>
-      <c r="F36" s="36"/>
+      <c r="A36" s="54" t="s">
+        <v>119</v>
+      </c>
+      <c r="B36" s="55"/>
+      <c r="C36" s="55"/>
+      <c r="D36" s="55"/>
+      <c r="E36" s="55"/>
+      <c r="F36" s="55"/>
       <c r="G36" s="5"/>
       <c r="H36" s="5"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A37" s="36"/>
-      <c r="B37" s="36"/>
-      <c r="C37" s="36"/>
-      <c r="D37" s="36"/>
-      <c r="E37" s="36"/>
-      <c r="F37" s="36"/>
+      <c r="A37" s="55"/>
+      <c r="B37" s="55"/>
+      <c r="C37" s="55"/>
+      <c r="D37" s="55"/>
+      <c r="E37" s="55"/>
+      <c r="F37" s="55"/>
       <c r="G37" s="5"/>
       <c r="H37" s="5"/>
     </row>
@@ -2141,7 +2183,29 @@
       <c r="H39" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="34">
+  <mergeCells count="38">
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="H7:H8"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="H13:H14"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="H29:H30"/>
+    <mergeCell ref="A36:F37"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="E3:E8"/>
+    <mergeCell ref="F3:F8"/>
+    <mergeCell ref="E9:E14"/>
+    <mergeCell ref="F9:F14"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="E23:E28"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="E29:E30"/>
     <mergeCell ref="C5:C8"/>
     <mergeCell ref="C33:C34"/>
     <mergeCell ref="A1:H1"/>
@@ -2158,24 +2222,6 @@
     <mergeCell ref="C19:C20"/>
     <mergeCell ref="C21:C22"/>
     <mergeCell ref="H15:H22"/>
-    <mergeCell ref="E3:E8"/>
-    <mergeCell ref="F3:F8"/>
-    <mergeCell ref="E9:E14"/>
-    <mergeCell ref="F9:F14"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="E23:E28"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="H29:H30"/>
-    <mergeCell ref="A36:F37"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="F33:F34"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2199,18 +2245,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>47</v>
@@ -2229,16 +2275,16 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="37">
+      <c r="A3" s="46">
         <v>1</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="C3" s="37" t="s">
+        <v>80</v>
+      </c>
+      <c r="C3" s="46" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="37" t="s">
+      <c r="D3" s="46" t="s">
         <v>7</v>
       </c>
       <c r="E3" s="12" t="s">
@@ -2249,26 +2295,26 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="37"/>
+      <c r="A4" s="46"/>
       <c r="B4" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="C4" s="37"/>
-      <c r="D4" s="37"/>
+        <v>81</v>
+      </c>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
       <c r="E4" s="12" t="s">
         <v>27</v>
       </c>
       <c r="F4" s="58"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="37"/>
+      <c r="A5" s="46"/>
       <c r="B5" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="C5" s="37" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5" s="46" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="37" t="s">
+      <c r="D5" s="46" t="s">
         <v>7</v>
       </c>
       <c r="E5" s="12" t="s">
@@ -2279,28 +2325,28 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="37"/>
+      <c r="A6" s="46"/>
       <c r="B6" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
+        <v>83</v>
+      </c>
+      <c r="C6" s="46"/>
+      <c r="D6" s="46"/>
       <c r="E6" s="12" t="s">
         <v>27</v>
       </c>
       <c r="F6" s="58"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="37">
+      <c r="A7" s="46">
         <v>2</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="C7" s="37" t="s">
+        <v>80</v>
+      </c>
+      <c r="C7" s="46" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="37" t="s">
+      <c r="D7" s="46" t="s">
         <v>7</v>
       </c>
       <c r="E7" s="12" t="s">
@@ -2311,26 +2357,26 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="37"/>
+      <c r="A8" s="46"/>
       <c r="B8" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="C8" s="37"/>
-      <c r="D8" s="37"/>
+        <v>81</v>
+      </c>
+      <c r="C8" s="46"/>
+      <c r="D8" s="46"/>
       <c r="E8" s="12" t="s">
         <v>27</v>
       </c>
       <c r="F8" s="58"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="37"/>
+      <c r="A9" s="46"/>
       <c r="B9" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="C9" s="37" t="s">
+        <v>82</v>
+      </c>
+      <c r="C9" s="46" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="37" t="s">
+      <c r="D9" s="46" t="s">
         <v>7</v>
       </c>
       <c r="E9" s="12" t="s">
@@ -2341,12 +2387,12 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="37"/>
+      <c r="A10" s="46"/>
       <c r="B10" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="C10" s="37"/>
-      <c r="D10" s="37"/>
+        <v>83</v>
+      </c>
+      <c r="C10" s="46"/>
+      <c r="D10" s="46"/>
       <c r="E10" s="12" t="s">
         <v>27</v>
       </c>
@@ -2390,57 +2436,57 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
-        <v>88</v>
-      </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
+      <c r="A1" s="36" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
       <c r="F1" s="6"/>
       <c r="G1" s="6"/>
     </row>
     <row r="2" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="59" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="E3" s="60" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="59"/>
       <c r="B4" s="14" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D4" s="14"/>
       <c r="E4" s="60"/>
@@ -2448,38 +2494,38 @@
     <row r="5" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="59"/>
       <c r="B5" s="14" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E5" s="60"/>
     </row>
     <row r="6" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B6" s="14"/>
       <c r="C6" s="11" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D6" s="14"/>
       <c r="E6" s="12"/>
     </row>
     <row r="7" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B7" s="14"/>
       <c r="C7" s="16" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D7" s="14"/>
       <c r="E7" s="15" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -2488,44 +2534,44 @@
       </c>
       <c r="B8" s="14"/>
       <c r="C8" s="17" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="D8" s="14"/>
       <c r="E8" s="12"/>
     </row>
     <row r="9" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B9" s="14"/>
       <c r="C9" s="14" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D9" s="14"/>
       <c r="E9" s="12"/>
     </row>
     <row r="10" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D10" s="14"/>
       <c r="E10" s="12"/>
     </row>
     <row r="11" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D11" s="14"/>
       <c r="E11" s="12"/>
@@ -2536,7 +2582,7 @@
       </c>
       <c r="B12" s="14"/>
       <c r="C12" s="14" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D12" s="14"/>
       <c r="E12" s="12"/>

</xml_diff>

<commit_message>
Refactor timer configurations; adjust prescaler and period values for improved timing accuracy, change PID parameters, Left back Right back wheel's PID parameters have been set properly. It's really a great success!!!
</commit_message>
<xml_diff>
--- a/参考资料/电气连接表.xlsx
+++ b/参考资料/电气连接表.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\STM32\Aks_SmartCar\Aks-SmartCar\参考资料\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AADD7727-6FA6-4631-8601-2633AAA7A1C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C11A0F9A-3714-4D15-B186-537D78B334A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{1220A042-B9C9-4738-A05B-507579105497}"/>
   </bookViews>
@@ -1771,7 +1771,7 @@
         <v>154</v>
       </c>
       <c r="G17" s="21" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H17" s="44"/>
     </row>
@@ -1789,7 +1789,7 @@
       <c r="E18" s="38"/>
       <c r="F18" s="37"/>
       <c r="G18" s="21" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H18" s="44"/>
     </row>
@@ -1851,7 +1851,7 @@
         <v>156</v>
       </c>
       <c r="G21" s="21" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H21" s="44"/>
       <c r="I21" s="53"/>
@@ -1870,7 +1870,7 @@
       <c r="E22" s="38"/>
       <c r="F22" s="37"/>
       <c r="G22" s="21" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H22" s="45"/>
       <c r="I22" s="53"/>

</xml_diff>

<commit_message>
Adjust timer prescaler and read period for improved timing accuracy; remove unused code
</commit_message>
<xml_diff>
--- a/参考资料/电气连接表.xlsx
+++ b/参考资料/电气连接表.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\STM32\Aks_SmartCar\Aks-SmartCar\参考资料\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C11A0F9A-3714-4D15-B186-537D78B334A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5147473-BFC9-4190-880C-9601C3D3B2B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{1220A042-B9C9-4738-A05B-507579105497}"/>
   </bookViews>
@@ -174,9 +174,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>PD3</t>
-  </si>
-  <si>
     <t>PD1</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -184,20 +181,11 @@
     <t>PD2</t>
   </si>
   <si>
-    <t>PD4</t>
-  </si>
-  <si>
     <t>PE1</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>PE2</t>
-  </si>
-  <si>
-    <t>PE3</t>
-  </si>
-  <si>
-    <t>PE4</t>
   </si>
   <si>
     <t>IN2</t>
@@ -649,6 +637,22 @@
   </si>
   <si>
     <t>JGB37-520电机编码器4RB</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PF14</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PF15</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PB0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PB1</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -990,6 +994,60 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -997,12 +1055,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1035,42 +1087,6 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1079,18 +1095,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1422,16 +1426,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="7" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="52" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
@@ -1441,7 +1445,7 @@
         <v>19</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D2" s="9" t="s">
         <v>8</v>
@@ -1456,7 +1460,7 @@
         <v>9</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -1464,25 +1468,25 @@
         <v>23</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="C3" s="39" t="s">
-        <v>114</v>
+        <v>58</v>
+      </c>
+      <c r="C3" s="55" t="s">
+        <v>110</v>
       </c>
       <c r="D3" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="46" t="s">
+      <c r="E3" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="47" t="s">
+      <c r="F3" s="38" t="s">
         <v>17</v>
       </c>
       <c r="G3" s="12" t="s">
         <v>11</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -1490,123 +1494,123 @@
         <v>24</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>63</v>
-      </c>
-      <c r="C4" s="40"/>
+        <v>59</v>
+      </c>
+      <c r="C4" s="56"/>
       <c r="D4" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="46"/>
-      <c r="F4" s="47"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="38"/>
       <c r="G4" s="12" t="s">
         <v>12</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B5" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="31" t="s">
-        <v>113</v>
+      <c r="C5" s="49" t="s">
+        <v>109</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="46"/>
-      <c r="F5" s="47"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="38"/>
       <c r="G5" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="61" t="s">
-        <v>149</v>
+      <c r="H5" s="31" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="32"/>
+      <c r="C6" s="50"/>
       <c r="D6" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="46"/>
-      <c r="F6" s="47"/>
+      <c r="E6" s="45"/>
+      <c r="F6" s="38"/>
       <c r="G6" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="H6" s="62"/>
+        <v>39</v>
+      </c>
+      <c r="H6" s="32"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
-        <v>35</v>
+        <v>153</v>
       </c>
       <c r="B7" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="32"/>
+      <c r="C7" s="50"/>
       <c r="D7" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="46"/>
-      <c r="F7" s="47"/>
+      <c r="E7" s="45"/>
+      <c r="F7" s="38"/>
       <c r="G7" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="61" t="s">
-        <v>150</v>
+      <c r="H7" s="31" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
-        <v>38</v>
+        <v>154</v>
       </c>
       <c r="B8" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="33"/>
+      <c r="C8" s="51"/>
       <c r="D8" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="46"/>
-      <c r="F8" s="47"/>
+      <c r="E8" s="45"/>
+      <c r="F8" s="38"/>
       <c r="G8" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="H8" s="62"/>
+      <c r="H8" s="32"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="26" t="s">
         <v>22</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>64</v>
-      </c>
-      <c r="C9" s="39" t="s">
-        <v>114</v>
+        <v>60</v>
+      </c>
+      <c r="C9" s="55" t="s">
+        <v>110</v>
       </c>
       <c r="D9" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="46" t="s">
+      <c r="E9" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="47" t="s">
+      <c r="F9" s="38" t="s">
         <v>18</v>
       </c>
       <c r="G9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -1614,284 +1618,284 @@
         <v>25</v>
       </c>
       <c r="B10" s="26" t="s">
-        <v>65</v>
-      </c>
-      <c r="C10" s="40"/>
+        <v>61</v>
+      </c>
+      <c r="C10" s="56"/>
       <c r="D10" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="E10" s="46"/>
-      <c r="F10" s="47"/>
+      <c r="E10" s="45"/>
+      <c r="F10" s="38"/>
       <c r="G10" s="12" t="s">
         <v>12</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="13" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B11" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="31" t="s">
-        <v>113</v>
+      <c r="C11" s="49" t="s">
+        <v>109</v>
       </c>
       <c r="D11" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E11" s="46"/>
-      <c r="F11" s="47"/>
+      <c r="E11" s="45"/>
+      <c r="F11" s="38"/>
       <c r="G11" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H11" s="63" t="s">
-        <v>151</v>
+      <c r="H11" s="33" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B12" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="32"/>
+      <c r="C12" s="50"/>
       <c r="D12" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="46"/>
-      <c r="F12" s="47"/>
+      <c r="E12" s="45"/>
+      <c r="F12" s="38"/>
       <c r="G12" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H12" s="64"/>
+      <c r="H12" s="34"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="13" t="s">
-        <v>41</v>
+        <v>155</v>
       </c>
       <c r="B13" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="32"/>
+      <c r="C13" s="50"/>
       <c r="D13" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E13" s="46"/>
-      <c r="F13" s="47"/>
+      <c r="E13" s="45"/>
+      <c r="F13" s="38"/>
       <c r="G13" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H13" s="61" t="s">
-        <v>152</v>
+      <c r="H13" s="31" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="13" t="s">
-        <v>42</v>
+        <v>156</v>
       </c>
       <c r="B14" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="33"/>
+      <c r="C14" s="51"/>
       <c r="D14" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E14" s="46"/>
-      <c r="F14" s="47"/>
+      <c r="E14" s="45"/>
+      <c r="F14" s="38"/>
       <c r="G14" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="H14" s="62"/>
+      <c r="H14" s="32"/>
     </row>
     <row r="15" spans="1:9" s="22" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="24" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B15" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="C15" s="41" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15" s="57" t="s">
+        <v>112</v>
+      </c>
+      <c r="D15" s="24" t="s">
+        <v>40</v>
+      </c>
+      <c r="E15" s="54" t="s">
+        <v>74</v>
+      </c>
+      <c r="F15" s="53" t="s">
+        <v>149</v>
+      </c>
+      <c r="G15" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="H15" s="59" t="s">
         <v>116</v>
       </c>
-      <c r="D15" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="E15" s="38" t="s">
-        <v>78</v>
-      </c>
-      <c r="F15" s="37" t="s">
-        <v>153</v>
-      </c>
-      <c r="G15" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="H15" s="43" t="s">
-        <v>120</v>
-      </c>
-      <c r="I15" s="53"/>
+      <c r="I15" s="37"/>
     </row>
     <row r="16" spans="1:9" s="22" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="24" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B16" s="24" t="s">
-        <v>128</v>
-      </c>
-      <c r="C16" s="42"/>
+        <v>124</v>
+      </c>
+      <c r="C16" s="58"/>
       <c r="D16" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="E16" s="38"/>
-      <c r="F16" s="37"/>
+        <v>40</v>
+      </c>
+      <c r="E16" s="54"/>
+      <c r="F16" s="53"/>
       <c r="G16" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="H16" s="44"/>
-      <c r="I16" s="53"/>
+        <v>57</v>
+      </c>
+      <c r="H16" s="60"/>
+      <c r="I16" s="37"/>
     </row>
     <row r="17" spans="1:9" s="22" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="24" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B17" s="24" t="s">
-        <v>73</v>
-      </c>
-      <c r="C17" s="41" t="s">
-        <v>117</v>
+        <v>69</v>
+      </c>
+      <c r="C17" s="57" t="s">
+        <v>113</v>
       </c>
       <c r="D17" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="E17" s="38"/>
-      <c r="F17" s="37" t="s">
-        <v>154</v>
+        <v>40</v>
+      </c>
+      <c r="E17" s="54"/>
+      <c r="F17" s="53" t="s">
+        <v>150</v>
       </c>
       <c r="G17" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="H17" s="44"/>
+        <v>57</v>
+      </c>
+      <c r="H17" s="60"/>
     </row>
     <row r="18" spans="1:9" s="22" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="24" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B18" s="24" t="s">
-        <v>124</v>
-      </c>
-      <c r="C18" s="42"/>
+        <v>120</v>
+      </c>
+      <c r="C18" s="58"/>
       <c r="D18" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="E18" s="38"/>
-      <c r="F18" s="37"/>
+        <v>40</v>
+      </c>
+      <c r="E18" s="54"/>
+      <c r="F18" s="53"/>
       <c r="G18" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="H18" s="44"/>
+        <v>56</v>
+      </c>
+      <c r="H18" s="60"/>
     </row>
     <row r="19" spans="1:9" s="22" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="24" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B19" s="24" t="s">
-        <v>76</v>
-      </c>
-      <c r="C19" s="41" t="s">
-        <v>123</v>
+        <v>72</v>
+      </c>
+      <c r="C19" s="57" t="s">
+        <v>119</v>
       </c>
       <c r="D19" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="E19" s="38"/>
-      <c r="F19" s="37" t="s">
-        <v>155</v>
+        <v>40</v>
+      </c>
+      <c r="E19" s="54"/>
+      <c r="F19" s="53" t="s">
+        <v>151</v>
       </c>
       <c r="G19" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="H19" s="44"/>
+        <v>56</v>
+      </c>
+      <c r="H19" s="60"/>
     </row>
     <row r="20" spans="1:9" s="22" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="24" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B20" s="24" t="s">
-        <v>77</v>
-      </c>
-      <c r="C20" s="42"/>
+        <v>73</v>
+      </c>
+      <c r="C20" s="58"/>
       <c r="D20" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="E20" s="38"/>
-      <c r="F20" s="37"/>
+        <v>40</v>
+      </c>
+      <c r="E20" s="54"/>
+      <c r="F20" s="53"/>
       <c r="G20" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="H20" s="44"/>
+        <v>57</v>
+      </c>
+      <c r="H20" s="60"/>
     </row>
     <row r="21" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="24" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B21" s="24" t="s">
-        <v>70</v>
-      </c>
-      <c r="C21" s="41" t="s">
-        <v>122</v>
+        <v>66</v>
+      </c>
+      <c r="C21" s="57" t="s">
+        <v>118</v>
       </c>
       <c r="D21" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="E21" s="38"/>
-      <c r="F21" s="37" t="s">
-        <v>156</v>
+        <v>40</v>
+      </c>
+      <c r="E21" s="54"/>
+      <c r="F21" s="53" t="s">
+        <v>152</v>
       </c>
       <c r="G21" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="H21" s="44"/>
-      <c r="I21" s="53"/>
+        <v>57</v>
+      </c>
+      <c r="H21" s="60"/>
+      <c r="I21" s="37"/>
     </row>
     <row r="22" spans="1:9" s="22" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="24" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B22" s="24" t="s">
-        <v>71</v>
-      </c>
-      <c r="C22" s="42"/>
+        <v>67</v>
+      </c>
+      <c r="C22" s="58"/>
       <c r="D22" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="E22" s="38"/>
-      <c r="F22" s="37"/>
+        <v>40</v>
+      </c>
+      <c r="E22" s="54"/>
+      <c r="F22" s="53"/>
       <c r="G22" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="H22" s="45"/>
-      <c r="I22" s="53"/>
+        <v>56</v>
+      </c>
+      <c r="H22" s="61"/>
+      <c r="I22" s="37"/>
     </row>
     <row r="23" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="13" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C23" s="30" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D23" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E23" s="46" t="s">
-        <v>45</v>
-      </c>
-      <c r="F23" s="47" t="s">
+      <c r="E23" s="45" t="s">
+        <v>41</v>
+      </c>
+      <c r="F23" s="38" t="s">
         <v>2</v>
       </c>
       <c r="G23" s="12" t="s">
@@ -1901,19 +1905,19 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="26" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B24" s="26" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C24" s="29" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D24" s="26" t="s">
-        <v>44</v>
-      </c>
-      <c r="E24" s="46"/>
-      <c r="F24" s="47"/>
+        <v>40</v>
+      </c>
+      <c r="E24" s="45"/>
+      <c r="F24" s="38"/>
       <c r="G24" s="12" t="s">
         <v>34</v>
       </c>
@@ -1921,19 +1925,19 @@
     </row>
     <row r="25" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="13" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C25" s="30" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D25" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E25" s="46"/>
-      <c r="F25" s="47" t="s">
+      <c r="E25" s="45"/>
+      <c r="F25" s="38" t="s">
         <v>3</v>
       </c>
       <c r="G25" s="12" t="s">
@@ -1943,19 +1947,19 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="26" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B26" s="26" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C26" s="29" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D26" s="26" t="s">
-        <v>44</v>
-      </c>
-      <c r="E26" s="46"/>
-      <c r="F26" s="47"/>
+        <v>40</v>
+      </c>
+      <c r="E26" s="45"/>
+      <c r="F26" s="38"/>
       <c r="G26" s="12" t="s">
         <v>34</v>
       </c>
@@ -1963,19 +1967,19 @@
     </row>
     <row r="27" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="13" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C27" s="30" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D27" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E27" s="46"/>
-      <c r="F27" s="47" t="s">
+      <c r="E27" s="45"/>
+      <c r="F27" s="38" t="s">
         <v>4</v>
       </c>
       <c r="G27" s="12" t="s">
@@ -1985,19 +1989,19 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="26" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B28" s="26" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C28" s="29" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D28" s="26" t="s">
-        <v>44</v>
-      </c>
-      <c r="E28" s="46"/>
-      <c r="F28" s="47"/>
+        <v>40</v>
+      </c>
+      <c r="E28" s="45"/>
+      <c r="F28" s="38"/>
       <c r="G28" s="12" t="s">
         <v>34</v>
       </c>
@@ -2005,160 +2009,160 @@
     </row>
     <row r="29" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="25" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B29" s="25" t="s">
-        <v>130</v>
-      </c>
-      <c r="C29" s="51" t="s">
-        <v>132</v>
+        <v>126</v>
+      </c>
+      <c r="C29" s="35" t="s">
+        <v>128</v>
       </c>
       <c r="D29" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="E29" s="50" t="s">
-        <v>55</v>
-      </c>
-      <c r="F29" s="49" t="s">
-        <v>54</v>
+      <c r="E29" s="48" t="s">
+        <v>51</v>
+      </c>
+      <c r="F29" s="47" t="s">
+        <v>50</v>
       </c>
       <c r="G29" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="H29" s="47" t="s">
-        <v>53</v>
+        <v>46</v>
+      </c>
+      <c r="H29" s="38" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="30" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="25" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B30" s="25" t="s">
-        <v>129</v>
-      </c>
-      <c r="C30" s="52"/>
+        <v>125</v>
+      </c>
+      <c r="C30" s="36"/>
       <c r="D30" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="E30" s="50"/>
-      <c r="F30" s="49"/>
+        <v>40</v>
+      </c>
+      <c r="E30" s="48"/>
+      <c r="F30" s="47"/>
       <c r="G30" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="H30" s="47"/>
+        <v>47</v>
+      </c>
+      <c r="H30" s="38"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="27" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B31" s="27" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D31" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="E31" s="48" t="s">
+      <c r="E31" s="46" t="s">
         <v>0</v>
       </c>
       <c r="F31" s="28" t="s">
         <v>1</v>
       </c>
       <c r="G31" s="12" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="H31" s="12"/>
     </row>
     <row r="32" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="27" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B32" s="27" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C32" s="27" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D32" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="E32" s="48"/>
+      <c r="E32" s="46"/>
       <c r="F32" s="28" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G32" s="12" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="H32" s="12"/>
     </row>
     <row r="33" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="20" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B33" s="20" t="s">
-        <v>133</v>
-      </c>
-      <c r="C33" s="34" t="s">
-        <v>131</v>
+        <v>129</v>
+      </c>
+      <c r="C33" s="41" t="s">
+        <v>127</v>
       </c>
       <c r="D33" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="E33" s="34" t="s">
-        <v>111</v>
-      </c>
-      <c r="F33" s="56" t="s">
-        <v>110</v>
+      <c r="E33" s="41" t="s">
+        <v>107</v>
+      </c>
+      <c r="F33" s="43" t="s">
+        <v>106</v>
       </c>
       <c r="G33" s="19" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H33" s="19"/>
     </row>
     <row r="34" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="20" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="C34" s="35"/>
+        <v>130</v>
+      </c>
+      <c r="C34" s="42"/>
       <c r="D34" s="20" t="s">
-        <v>44</v>
-      </c>
-      <c r="E34" s="35"/>
-      <c r="F34" s="57"/>
+        <v>40</v>
+      </c>
+      <c r="E34" s="42"/>
+      <c r="F34" s="44"/>
       <c r="G34" s="19" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="H34" s="19"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="8" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A36" s="54" t="s">
-        <v>119</v>
-      </c>
-      <c r="B36" s="55"/>
-      <c r="C36" s="55"/>
-      <c r="D36" s="55"/>
-      <c r="E36" s="55"/>
-      <c r="F36" s="55"/>
+      <c r="A36" s="39" t="s">
+        <v>115</v>
+      </c>
+      <c r="B36" s="40"/>
+      <c r="C36" s="40"/>
+      <c r="D36" s="40"/>
+      <c r="E36" s="40"/>
+      <c r="F36" s="40"/>
       <c r="G36" s="5"/>
       <c r="H36" s="5"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A37" s="55"/>
-      <c r="B37" s="55"/>
-      <c r="C37" s="55"/>
-      <c r="D37" s="55"/>
-      <c r="E37" s="55"/>
-      <c r="F37" s="55"/>
+      <c r="A37" s="40"/>
+      <c r="B37" s="40"/>
+      <c r="C37" s="40"/>
+      <c r="D37" s="40"/>
+      <c r="E37" s="40"/>
+      <c r="F37" s="40"/>
       <c r="G37" s="5"/>
       <c r="H37" s="5"/>
     </row>
@@ -2184,30 +2188,6 @@
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="H7:H8"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="H13:H14"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="H29:H30"/>
-    <mergeCell ref="A36:F37"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="E3:E8"/>
-    <mergeCell ref="F3:F8"/>
-    <mergeCell ref="E9:E14"/>
-    <mergeCell ref="F9:F14"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="E23:E28"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="C5:C8"/>
-    <mergeCell ref="C33:C34"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="F15:F16"/>
     <mergeCell ref="F17:F18"/>
@@ -2222,6 +2202,30 @@
     <mergeCell ref="C19:C20"/>
     <mergeCell ref="C21:C22"/>
     <mergeCell ref="H15:H22"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="H29:H30"/>
+    <mergeCell ref="A36:F37"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="E23:E28"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="C33:C34"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="H7:H8"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="H13:H14"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="E3:E8"/>
+    <mergeCell ref="F3:F8"/>
+    <mergeCell ref="E9:E14"/>
+    <mergeCell ref="F9:F14"/>
+    <mergeCell ref="C5:C8"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2245,21 +2249,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="36" t="s">
-        <v>46</v>
-      </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
+      <c r="A1" s="52" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C2" s="9" t="s">
         <v>29</v>
@@ -2275,128 +2279,128 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="46">
+      <c r="A3" s="45">
         <v>1</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="C3" s="46" t="s">
+        <v>76</v>
+      </c>
+      <c r="C3" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="46" t="s">
+      <c r="D3" s="45" t="s">
         <v>7</v>
       </c>
       <c r="E3" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="58" t="s">
+      <c r="F3" s="62" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="46"/>
+      <c r="A4" s="45"/>
       <c r="B4" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
+        <v>77</v>
+      </c>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
       <c r="E4" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="58"/>
+      <c r="F4" s="62"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="46"/>
+      <c r="A5" s="45"/>
       <c r="B5" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="C5" s="46" t="s">
+        <v>78</v>
+      </c>
+      <c r="C5" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="46" t="s">
+      <c r="D5" s="45" t="s">
         <v>7</v>
       </c>
       <c r="E5" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="F5" s="58" t="s">
+      <c r="F5" s="62" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="46"/>
+      <c r="A6" s="45"/>
       <c r="B6" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="C6" s="46"/>
-      <c r="D6" s="46"/>
+        <v>79</v>
+      </c>
+      <c r="C6" s="45"/>
+      <c r="D6" s="45"/>
       <c r="E6" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="F6" s="58"/>
+      <c r="F6" s="62"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="46">
+      <c r="A7" s="45">
         <v>2</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="C7" s="46" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="46" t="s">
+      <c r="D7" s="45" t="s">
         <v>7</v>
       </c>
       <c r="E7" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="F7" s="58" t="s">
+      <c r="F7" s="62" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="46"/>
+      <c r="A8" s="45"/>
       <c r="B8" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="C8" s="46"/>
-      <c r="D8" s="46"/>
+        <v>77</v>
+      </c>
+      <c r="C8" s="45"/>
+      <c r="D8" s="45"/>
       <c r="E8" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="F8" s="58"/>
+      <c r="F8" s="62"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="46"/>
+      <c r="A9" s="45"/>
       <c r="B9" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="C9" s="46" t="s">
+        <v>78</v>
+      </c>
+      <c r="C9" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="46" t="s">
+      <c r="D9" s="45" t="s">
         <v>7</v>
       </c>
       <c r="E9" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="58" t="s">
+      <c r="F9" s="62" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="46"/>
+      <c r="A10" s="45"/>
       <c r="B10" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="C10" s="46"/>
-      <c r="D10" s="46"/>
+        <v>79</v>
+      </c>
+      <c r="C10" s="45"/>
+      <c r="D10" s="45"/>
       <c r="E10" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="F10" s="58"/>
+      <c r="F10" s="62"/>
     </row>
   </sheetData>
   <mergeCells count="15">
@@ -2436,96 +2440,96 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="36" t="s">
-        <v>84</v>
-      </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
+      <c r="A1" s="52" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
       <c r="F1" s="6"/>
       <c r="G1" s="6"/>
     </row>
     <row r="2" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="59" t="s">
-        <v>109</v>
+      <c r="A3" s="63" t="s">
+        <v>105</v>
       </c>
       <c r="B3" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="E3" s="64" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="63"/>
+      <c r="B4" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="D4" s="14"/>
+      <c r="E4" s="64"/>
+    </row>
+    <row r="5" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="63"/>
+      <c r="B5" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="D5" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="C3" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="E3" s="60" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="59"/>
-      <c r="B4" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>101</v>
-      </c>
-      <c r="D4" s="14"/>
-      <c r="E4" s="60"/>
-    </row>
-    <row r="5" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="59"/>
-      <c r="B5" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="C5" s="17" t="s">
-        <v>97</v>
-      </c>
-      <c r="D5" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="E5" s="60"/>
+      <c r="E5" s="64"/>
     </row>
     <row r="6" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B6" s="14"/>
       <c r="C6" s="11" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="D6" s="14"/>
       <c r="E6" s="12"/>
     </row>
     <row r="7" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B7" s="14"/>
       <c r="C7" s="16" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D7" s="14"/>
       <c r="E7" s="15" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.3">
@@ -2534,44 +2538,44 @@
       </c>
       <c r="B8" s="14"/>
       <c r="C8" s="17" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D8" s="14"/>
       <c r="E8" s="12"/>
     </row>
     <row r="9" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B9" s="14"/>
       <c r="C9" s="14" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D9" s="14"/>
       <c r="E9" s="12"/>
     </row>
     <row r="10" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D10" s="14"/>
       <c r="E10" s="12"/>
     </row>
     <row r="11" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D11" s="14"/>
       <c r="E11" s="12"/>
@@ -2582,7 +2586,7 @@
       </c>
       <c r="B12" s="14"/>
       <c r="C12" s="14" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D12" s="14"/>
       <c r="E12" s="12"/>

</xml_diff>